<commit_message>
Fixing error in sheets containing TYNDP collection and adding IE-FR and NO2-NL lines
</commit_message>
<xml_diff>
--- a/analysis/preprocessing/20231103-TYNDP2024-GRID.xlsx
+++ b/analysis/preprocessing/20231103-TYNDP2024-GRID.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Content" sheetId="1" state="visible" r:id="rId3"/>
@@ -1869,7 +1869,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1989,12 +1989,6 @@
       <name val="Calibri"/>
       <family val="0"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -2061,7 +2055,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2128,10 +2122,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2243,9 +2233,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>131400</xdr:colOff>
+      <xdr:colOff>131040</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>140760</xdr:rowOff>
+      <xdr:rowOff>140400</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2255,7 +2245,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="231840" y="181080"/>
-          <a:ext cx="13964040" cy="9551520"/>
+          <a:ext cx="13963680" cy="9551160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2716,7 +2706,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>capacities across Europe, according to the data that member TSOs have for 2030. The aforementioned year </a:t>
+            <a:t>capacities across Europe, according to the data that member TSOs have for 2030. The aforementioned </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
@@ -2727,7 +2717,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>is the only one for which a reference grid is provided, as 2030 is the starting point for the DE/GA scenarios. </a:t>
+            <a:t>year is the only one for which a reference grid is provided, as 2030 is the starting point for the DE/GA </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
@@ -2738,7 +2728,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>After 2030, investment can happen in transmission candidate projects, which are gathered in a separate </a:t>
+            <a:t>scenarios. After 2030, investment can happen in transmission candidate projects, which are gathered in a </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
@@ -2749,7 +2739,7 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>file.</a:t>
+            <a:t>separate file.</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -3558,9 +3548,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>125640</xdr:colOff>
+      <xdr:colOff>125280</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>16920</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -3570,7 +3560,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10833840" y="343080"/>
-          <a:ext cx="5774040" cy="3293280"/>
+          <a:ext cx="5773680" cy="3292920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3795,9 +3785,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>464760</xdr:colOff>
+      <xdr:colOff>464400</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>55080</xdr:rowOff>
+      <xdr:rowOff>54720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -3807,7 +3797,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5157360" y="238320"/>
-          <a:ext cx="5419080" cy="3074400"/>
+          <a:ext cx="5418720" cy="3074040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4027,14 +4017,14 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>504720</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>142920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>137520</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>32400</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -4044,7 +4034,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9137520" y="504720"/>
-          <a:ext cx="6359400" cy="6405120"/>
+          <a:ext cx="6359040" cy="6404760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4716,9 +4706,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>318240</xdr:colOff>
+      <xdr:colOff>317880</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>148680</xdr:rowOff>
+      <xdr:rowOff>148320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -4727,8 +4717,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7358400" y="133200"/>
-          <a:ext cx="6393960" cy="5305680"/>
+          <a:off x="7358760" y="133200"/>
+          <a:ext cx="6393960" cy="5305320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4811,7 +4801,18 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>This file gathers the expansion candidates for hydrogen transmission across Europe, according to the data that member TSOs provided for the time horizon between 2035 and 2050.</a:t>
+            <a:t>This file gathers the expansion candidates for hydrogen transmission across Europe, according to </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>the data that member TSOs provided for the time horizon between 2035 and 2050.</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -4846,7 +4847,51 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>In essence, the hydrogen candidate projects that are made available in 2030 are associated with ENTSOG's "low infrastructure level" - a pre-defined level of the hydrogen transmission grid accounting for the cross-border interconnection projects with higher probability of getting commissioned. On the other hand, the projects available for expansion after 2040 are assocaited with ENTSOG's "high infrastructure level", where less certain candidates are also accounted for.</a:t>
+            <a:t>In essence, the hydrogen candidate projects that are made available in 2030 are associated with </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>ENTSOG's "low infrastructure level" - a pre-defined level of the hydrogen transmission grid </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>accounting for the cross-border interconnection projects with higher probability of getting </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>commissioned. On the other hand, the projects available for expansion after 2040 are assocaited </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>with ENTSOG's "high infrastructure level", where less certain candidates are also accounted for.</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -4904,7 +4949,18 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>- Border --- the border on which the interconnector is found (note that the nodes linked by interconnector keep the ISO2 naming convention)</a:t>
+            <a:t>- Border --- the border on which the interconnector is found (note that the nodes linked by </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>interconnector keep the ISO2 naming convention)</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -4973,7 +5029,18 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>- Year --- the year in which the project becomes available for the expansion planning problem, i.e., one of the five target years modelled (2030, 2035, 2040, 2045, 2050)</a:t>
+            <a:t>- Year --- the year in which the project becomes available for the expansion planning problem, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>i.e., one of the five target years modelled (2030, 2035, 2040, 2045, 2050)</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -5019,7 +5086,18 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>- Direct Capacity Increase --- incremental capacity of interconnector in the direction listed in the index, e.g., AT-IT</a:t>
+            <a:t>- Direct Capacity Increase --- incremental capacity of interconnector in the direction listed in the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>index, e.g., AT-IT</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -5042,7 +5120,18 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>- Indirect Capacity Increase --- increamental capacity of interconnector in the direction opposite to the one found in the index, e.g., IT-AT</a:t>
+            <a:t>- Indirect Capacity Increase --- increamental capacity of interconnector in the direction opposite </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>to the one found in the index, e.g., IT-AT</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -5103,7 +5192,29 @@
               <a:uFillTx/>
               <a:latin typeface="Calibri"/>
             </a:rPr>
-            <a:t>The expansion methodology considers all the listed candidates as discrete investment decisions, however the solution method assumes a linear relaxation, i.e., any share of the installed capacity in the [0,1] interval can be part of the expansion planning problem solution.</a:t>
+            <a:t>The expansion methodology considers all the listed candidates as discrete investment decisions, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>however the solution method assumes a linear relaxation, i.e., any share of the installed </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>capacity in the [0,1] interval can be part of the expansion planning problem solution.</a:t>
           </a:r>
           <a:endParaRPr lang="en-DK" sz="1100" b="0" u="none" strike="noStrike">
             <a:effectLst/>
@@ -7479,7 +7590,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+  <sheetPr filterMode="true">
     <tabColor rgb="FF5B9BD5"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -7548,7 +7659,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
         <v>201</v>
       </c>
@@ -7600,7 +7711,7 @@
         <v>316.7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>204</v>
       </c>
@@ -7652,7 +7763,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>209</v>
       </c>
@@ -7756,7 +7867,7 @@
         <v>1649</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>216</v>
       </c>
@@ -7834,7 +7945,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
         <v>222</v>
       </c>
@@ -8328,7 +8439,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
         <v>256</v>
       </c>
@@ -8432,7 +8543,7 @@
         <v>87.55</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
         <v>263</v>
       </c>
@@ -8614,7 +8725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
         <v>276</v>
       </c>
@@ -8744,7 +8855,7 @@
         <v>1489.92</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
         <v>281</v>
       </c>
@@ -8770,7 +8881,7 @@
         <v>2285.92</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
         <v>282</v>
       </c>
@@ -8874,7 +8985,7 @@
         <v>547.24</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
         <v>286</v>
       </c>
@@ -8900,7 +9011,7 @@
         <v>656.3</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
         <v>287</v>
       </c>
@@ -8952,7 +9063,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
         <v>289</v>
       </c>
@@ -8978,7 +9089,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
         <v>290</v>
       </c>
@@ -9004,7 +9115,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="s">
         <v>291</v>
       </c>
@@ -9082,7 +9193,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
         <v>294</v>
       </c>
@@ -9108,7 +9219,7 @@
         <v>2617</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
         <v>295</v>
       </c>
@@ -9134,7 +9245,7 @@
         <v>110.5</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="s">
         <v>296</v>
       </c>
@@ -9160,7 +9271,7 @@
         <v>222.7</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="s">
         <v>297</v>
       </c>
@@ -9186,7 +9297,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="s">
         <v>298</v>
       </c>
@@ -9290,7 +9401,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
         <v>302</v>
       </c>
@@ -9316,7 +9427,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
         <v>303</v>
       </c>
@@ -9342,7 +9453,7 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="9" t="s">
         <v>304</v>
       </c>
@@ -9368,7 +9479,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
         <v>305</v>
       </c>
@@ -9394,7 +9505,7 @@
         <v>2977</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="9" t="s">
         <v>306</v>
       </c>
@@ -9420,7 +9531,7 @@
         <v>4065</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="9" t="s">
         <v>307</v>
       </c>
@@ -9446,7 +9557,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="9" t="s">
         <v>309</v>
       </c>
@@ -9472,7 +9583,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="9" t="s">
         <v>310</v>
       </c>
@@ -9498,7 +9609,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="9" t="s">
         <v>311</v>
       </c>
@@ -9628,7 +9739,7 @@
         <v>2540</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="9" t="s">
         <v>316</v>
       </c>
@@ -9654,7 +9765,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="9" t="s">
         <v>317</v>
       </c>
@@ -9680,7 +9791,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="9" t="s">
         <v>318</v>
       </c>
@@ -9706,7 +9817,7 @@
         <v>347.8</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="9" t="s">
         <v>319</v>
       </c>
@@ -9732,7 +9843,7 @@
         <v>477.8</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="9" t="s">
         <v>320</v>
       </c>
@@ -9758,7 +9869,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="9" t="s">
         <v>321</v>
       </c>
@@ -9888,7 +9999,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="9" t="s">
         <v>328</v>
       </c>
@@ -9992,7 +10103,7 @@
         <v>2075</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="9" t="s">
         <v>333</v>
       </c>
@@ -10018,7 +10129,7 @@
         <v>2125</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="9" t="s">
         <v>334</v>
       </c>
@@ -10044,7 +10155,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="9" t="s">
         <v>335</v>
       </c>
@@ -10070,7 +10181,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="9" t="s">
         <v>336</v>
       </c>
@@ -10096,7 +10207,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="9" t="s">
         <v>338</v>
       </c>
@@ -10122,7 +10233,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="9" t="s">
         <v>339</v>
       </c>
@@ -10148,7 +10259,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="9" t="s">
         <v>340</v>
       </c>
@@ -10174,7 +10285,7 @@
         <v>92.8</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="9" t="s">
         <v>341</v>
       </c>
@@ -10200,7 +10311,7 @@
         <v>47.7</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="9" t="s">
         <v>342</v>
       </c>
@@ -10226,7 +10337,7 @@
         <v>77.7</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="9" t="s">
         <v>343</v>
       </c>
@@ -10252,7 +10363,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="9" t="s">
         <v>344</v>
       </c>
@@ -10278,7 +10389,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="9" t="s">
         <v>345</v>
       </c>
@@ -10304,7 +10415,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="9" t="s">
         <v>346</v>
       </c>
@@ -10382,7 +10493,7 @@
         <v>499.18</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="9" t="s">
         <v>349</v>
       </c>
@@ -10434,7 +10545,7 @@
         <v>866.4</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="9" t="s">
         <v>351</v>
       </c>
@@ -10460,7 +10571,7 @@
         <v>1703.05</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="9" t="s">
         <v>352</v>
       </c>
@@ -10486,7 +10597,7 @@
         <v>18.86</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="9" t="s">
         <v>353</v>
       </c>
@@ -10512,7 +10623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="9" t="s">
         <v>354</v>
       </c>
@@ -10538,7 +10649,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="9" t="s">
         <v>355</v>
       </c>
@@ -10564,7 +10675,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="9" t="s">
         <v>356</v>
       </c>
@@ -10590,7 +10701,7 @@
         <v>132.1</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="9" t="s">
         <v>357</v>
       </c>
@@ -10616,7 +10727,7 @@
         <v>36.88</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="9" t="s">
         <v>358</v>
       </c>
@@ -10642,7 +10753,7 @@
         <v>29.46</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="9" t="s">
         <v>359</v>
       </c>
@@ -10668,7 +10779,7 @@
         <v>54.58</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="9" t="s">
         <v>360</v>
       </c>
@@ -10694,7 +10805,7 @@
         <v>62.48</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="9" t="s">
         <v>361</v>
       </c>
@@ -10720,7 +10831,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="9" t="s">
         <v>362</v>
       </c>
@@ -10746,7 +10857,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="9" t="s">
         <v>363</v>
       </c>
@@ -10772,7 +10883,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="9" t="s">
         <v>364</v>
       </c>
@@ -10798,7 +10909,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="9" t="s">
         <v>365</v>
       </c>
@@ -10824,7 +10935,7 @@
         <v>283.44</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="9" t="s">
         <v>366</v>
       </c>
@@ -10850,7 +10961,7 @@
         <v>283.44</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="9" t="s">
         <v>367</v>
       </c>
@@ -10876,7 +10987,7 @@
         <v>110.8</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="9" t="s">
         <v>368</v>
       </c>
@@ -10902,7 +11013,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="9" t="s">
         <v>369</v>
       </c>
@@ -10928,7 +11039,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="9" t="s">
         <v>370</v>
       </c>
@@ -10954,7 +11065,7 @@
         <v>3243</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="9" t="s">
         <v>371</v>
       </c>
@@ -10980,7 +11091,7 @@
         <v>3244</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="9" t="s">
         <v>372</v>
       </c>
@@ -11006,7 +11117,7 @@
         <v>3245</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="9" t="s">
         <v>373</v>
       </c>
@@ -11032,7 +11143,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="9" t="s">
         <v>375</v>
       </c>
@@ -11058,7 +11169,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="9" t="s">
         <v>376</v>
       </c>
@@ -11084,7 +11195,7 @@
         <v>345.3</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="9" t="s">
         <v>377</v>
       </c>
@@ -11162,7 +11273,7 @@
         <v>384.3</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="9" t="s">
         <v>381</v>
       </c>
@@ -11188,7 +11299,7 @@
         <v>385.3</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="9" t="s">
         <v>382</v>
       </c>
@@ -11214,7 +11325,7 @@
         <v>386.3</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="9" t="s">
         <v>383</v>
       </c>
@@ -11240,7 +11351,7 @@
         <v>387.3</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="9" t="s">
         <v>384</v>
       </c>
@@ -11266,7 +11377,7 @@
         <v>388.3</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="9" t="s">
         <v>385</v>
       </c>
@@ -11292,7 +11403,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="9" t="s">
         <v>386</v>
       </c>
@@ -11318,7 +11429,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="9" t="s">
         <v>387</v>
       </c>
@@ -11344,7 +11455,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="9" t="s">
         <v>388</v>
       </c>
@@ -11370,7 +11481,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="9" t="s">
         <v>389</v>
       </c>
@@ -11396,7 +11507,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="9" t="s">
         <v>390</v>
       </c>
@@ -11422,7 +11533,7 @@
         <v>478.6</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="9" t="s">
         <v>391</v>
       </c>
@@ -11448,7 +11559,7 @@
         <v>479.6</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="9" t="s">
         <v>392</v>
       </c>
@@ -11474,7 +11585,7 @@
         <v>480.6</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="9" t="s">
         <v>393</v>
       </c>
@@ -11500,7 +11611,7 @@
         <v>481.6</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="9" t="s">
         <v>394</v>
       </c>
@@ -11526,7 +11637,7 @@
         <v>482.6</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="9" t="s">
         <v>395</v>
       </c>
@@ -11552,7 +11663,7 @@
         <v>483.6</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="9" t="s">
         <v>396</v>
       </c>
@@ -11578,7 +11689,7 @@
         <v>3246</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="9" t="s">
         <v>397</v>
       </c>
@@ -11604,7 +11715,7 @@
         <v>3247</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="9" t="s">
         <v>398</v>
       </c>
@@ -11630,7 +11741,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="9" t="s">
         <v>399</v>
       </c>
@@ -11708,7 +11819,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="9" t="s">
         <v>402</v>
       </c>
@@ -11734,7 +11845,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="9" t="s">
         <v>403</v>
       </c>
@@ -11760,7 +11871,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="9" t="s">
         <v>404</v>
       </c>
@@ -11838,7 +11949,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="9" t="s">
         <v>407</v>
       </c>
@@ -11864,7 +11975,7 @@
         <v>3250</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="9" t="s">
         <v>408</v>
       </c>
@@ -12020,7 +12131,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="9" t="s">
         <v>414</v>
       </c>
@@ -12072,7 +12183,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="9" t="s">
         <v>416</v>
       </c>
@@ -12098,7 +12209,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="9" t="s">
         <v>417</v>
       </c>
@@ -12150,7 +12261,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="9" t="s">
         <v>420</v>
       </c>
@@ -12202,7 +12313,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="9" t="s">
         <v>422</v>
       </c>
@@ -12254,7 +12365,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="9" t="s">
         <v>424</v>
       </c>
@@ -12280,7 +12391,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="9" t="s">
         <v>425</v>
       </c>
@@ -12306,7 +12417,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="9" t="s">
         <v>426</v>
       </c>
@@ -12332,7 +12443,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="9" t="s">
         <v>427</v>
       </c>
@@ -12358,7 +12469,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="9" t="s">
         <v>428</v>
       </c>
@@ -12384,7 +12495,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="9" t="s">
         <v>429</v>
       </c>
@@ -12410,7 +12521,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="9" t="s">
         <v>430</v>
       </c>
@@ -12436,7 +12547,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="9" t="s">
         <v>431</v>
       </c>
@@ -12462,7 +12573,7 @@
         <v>1700</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="9" t="s">
         <v>432</v>
       </c>
@@ -12488,7 +12599,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="9" t="s">
         <v>433</v>
       </c>
@@ -12514,7 +12625,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="9" t="s">
         <v>434</v>
       </c>
@@ -12540,7 +12651,7 @@
         <v>118.75</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="9" t="s">
         <v>435</v>
       </c>
@@ -12566,7 +12677,7 @@
         <v>410.4</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="9" t="s">
         <v>436</v>
       </c>
@@ -12592,7 +12703,7 @@
         <v>624.6</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="9" t="s">
         <v>437</v>
       </c>
@@ -12618,7 +12729,7 @@
         <v>89.45</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="9" t="s">
         <v>438</v>
       </c>
@@ -12644,7 +12755,7 @@
         <v>124.23</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="9" t="s">
         <v>439</v>
       </c>
@@ -12800,7 +12911,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="9" t="s">
         <v>445</v>
       </c>
@@ -12826,7 +12937,7 @@
         <v>1939</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="9" t="s">
         <v>446</v>
       </c>
@@ -12852,7 +12963,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="9" t="s">
         <v>447</v>
       </c>
@@ -12878,7 +12989,7 @@
         <v>478.18</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="9" t="s">
         <v>448</v>
       </c>
@@ -12904,7 +13015,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="9" t="s">
         <v>449</v>
       </c>
@@ -12930,7 +13041,7 @@
         <v>441.5</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="9" t="s">
         <v>450</v>
       </c>
@@ -13086,7 +13197,7 @@
         <v>430.28</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="9" t="s">
         <v>456</v>
       </c>
@@ -13112,7 +13223,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="9" t="s">
         <v>457</v>
       </c>
@@ -13138,7 +13249,7 @@
         <v>1850</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="9" t="s">
         <v>458</v>
       </c>
@@ -13164,7 +13275,7 @@
         <v>54.82</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="9" t="s">
         <v>459</v>
       </c>
@@ -13190,7 +13301,7 @@
         <v>83.5</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="9" t="s">
         <v>460</v>
       </c>
@@ -13216,7 +13327,7 @@
         <v>95.34</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="9" t="s">
         <v>461</v>
       </c>
@@ -13242,7 +13353,7 @@
         <v>144.78</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="9" t="s">
         <v>462</v>
       </c>
@@ -13268,7 +13379,7 @@
         <v>2600</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="9" t="s">
         <v>463</v>
       </c>
@@ -13294,7 +13405,7 @@
         <v>2610</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="9" t="s">
         <v>464</v>
       </c>
@@ -13320,7 +13431,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="9" t="s">
         <v>466</v>
       </c>
@@ -13346,7 +13457,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="9" t="s">
         <v>467</v>
       </c>
@@ -13372,7 +13483,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="9" t="s">
         <v>468</v>
       </c>
@@ -13398,7 +13509,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="9" t="s">
         <v>469</v>
       </c>
@@ -13424,7 +13535,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="9" t="s">
         <v>470</v>
       </c>
@@ -13450,7 +13561,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="9" t="s">
         <v>471</v>
       </c>
@@ -13476,7 +13587,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="9" t="s">
         <v>472</v>
       </c>
@@ -13502,7 +13613,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="9" t="s">
         <v>473</v>
       </c>
@@ -13528,7 +13639,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="9" t="s">
         <v>474</v>
       </c>
@@ -13554,7 +13665,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="9" t="s">
         <v>475</v>
       </c>
@@ -13580,7 +13691,7 @@
         <v>1640</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="9" t="s">
         <v>476</v>
       </c>
@@ -13606,7 +13717,7 @@
         <v>1690</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="9" t="s">
         <v>477</v>
       </c>
@@ -13632,7 +13743,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="9" t="s">
         <v>478</v>
       </c>
@@ -13658,7 +13769,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="9" t="s">
         <v>479</v>
       </c>
@@ -13684,7 +13795,7 @@
         <v>149.01</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="9" t="s">
         <v>480</v>
       </c>
@@ -13710,7 +13821,7 @@
         <v>248.9</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="9" t="s">
         <v>481</v>
       </c>
@@ -13736,7 +13847,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="9" t="s">
         <v>482</v>
       </c>
@@ -13762,7 +13873,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="9" t="s">
         <v>483</v>
       </c>
@@ -13788,7 +13899,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="9" t="s">
         <v>484</v>
       </c>
@@ -13814,7 +13925,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="9" t="s">
         <v>485</v>
       </c>
@@ -13840,7 +13951,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="9" t="s">
         <v>486</v>
       </c>
@@ -14235,7 +14346,14 @@
       <c r="H261" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H261"/>
+  <autoFilter ref="A1:H261">
+    <filterColumn colId="3">
+      <filters blank="1">
+        <filter val="2030"/>
+        <filter val="2035"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.3"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -20855,8 +20973,8 @@
         <v>607</v>
       </c>
       <c r="E144" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B3</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C2</f>
+        <v>600</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20875,8 +20993,8 @@
         <v>607</v>
       </c>
       <c r="E145" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B4</f>
-        <v>500</v>
+        <f aca="false">'1. Elec Ref Grid'!C3</f>
+        <v>400</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20895,8 +21013,8 @@
         <v>607</v>
       </c>
       <c r="E146" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B5</f>
-        <v>250</v>
+        <f aca="false">'1. Elec Ref Grid'!C4</f>
+        <v>500</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20915,8 +21033,8 @@
         <v>607</v>
       </c>
       <c r="E147" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B6</f>
-        <v>1200</v>
+        <f aca="false">'1. Elec Ref Grid'!C5</f>
+        <v>250</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20935,8 +21053,8 @@
         <v>607</v>
       </c>
       <c r="E148" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B7</f>
-        <v>900</v>
+        <f aca="false">'1. Elec Ref Grid'!C6</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20955,8 +21073,8 @@
         <v>607</v>
       </c>
       <c r="E149" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B8</f>
-        <v>7500</v>
+        <f aca="false">'1. Elec Ref Grid'!C7</f>
+        <v>900</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20975,8 +21093,8 @@
         <v>607</v>
       </c>
       <c r="E150" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B9</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C8</f>
+        <v>7500</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20995,8 +21113,8 @@
         <v>607</v>
       </c>
       <c r="E151" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B10</f>
-        <v>875</v>
+        <f aca="false">'1. Elec Ref Grid'!C9</f>
+        <v>800</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21015,8 +21133,8 @@
         <v>607</v>
       </c>
       <c r="E152" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B11</f>
-        <v>950</v>
+        <f aca="false">'1. Elec Ref Grid'!C10</f>
+        <v>695</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21035,8 +21153,8 @@
         <v>607</v>
       </c>
       <c r="E153" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B12</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C11</f>
+        <v>950</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21055,8 +21173,8 @@
         <v>607</v>
       </c>
       <c r="E154" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B13</f>
-        <v>900</v>
+        <f aca="false">'1. Elec Ref Grid'!C12</f>
+        <v>0</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21075,8 +21193,8 @@
         <v>607</v>
       </c>
       <c r="E155" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B14</f>
-        <v>500</v>
+        <f aca="false">'1. Elec Ref Grid'!C13</f>
+        <v>800</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21095,8 +21213,8 @@
         <v>607</v>
       </c>
       <c r="E156" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B15</f>
-        <v>1640</v>
+        <f aca="false">'1. Elec Ref Grid'!C14</f>
+        <v>500</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21115,8 +21233,8 @@
         <v>607</v>
       </c>
       <c r="E157" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B16</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C15</f>
+        <v>1680</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21135,8 +21253,8 @@
         <v>607</v>
       </c>
       <c r="E158" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B17</f>
-        <v>2800</v>
+        <f aca="false">'1. Elec Ref Grid'!C16</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21155,8 +21273,8 @@
         <v>607</v>
       </c>
       <c r="E159" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B18</f>
-        <v>380</v>
+        <f aca="false">'1. Elec Ref Grid'!C17</f>
+        <v>4300</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21175,8 +21293,8 @@
         <v>607</v>
       </c>
       <c r="E160" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B19</f>
-        <v>300</v>
+        <f aca="false">'1. Elec Ref Grid'!C18</f>
+        <v>0</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21195,8 +21313,8 @@
         <v>607</v>
       </c>
       <c r="E161" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B20</f>
-        <v>3400</v>
+        <f aca="false">'1. Elec Ref Grid'!C19</f>
+        <v>180</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21215,8 +21333,8 @@
         <v>607</v>
       </c>
       <c r="E162" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B21</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C20</f>
+        <v>3400</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21235,8 +21353,8 @@
         <v>607</v>
       </c>
       <c r="E163" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B22</f>
-        <v>1700</v>
+        <f aca="false">'1. Elec Ref Grid'!C21</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21255,8 +21373,8 @@
         <v>607</v>
       </c>
       <c r="E164" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B23</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C22</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21275,8 +21393,8 @@
         <v>607</v>
       </c>
       <c r="E165" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B24</f>
-        <v>2190</v>
+        <f aca="false">'1. Elec Ref Grid'!C23</f>
+        <v>400</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21295,8 +21413,8 @@
         <v>607</v>
       </c>
       <c r="E166" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B25</f>
-        <v>380</v>
+        <f aca="false">'1. Elec Ref Grid'!C24</f>
+        <v>2190</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21315,8 +21433,8 @@
         <v>607</v>
       </c>
       <c r="E167" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B26</f>
-        <v>900</v>
+        <f aca="false">'1. Elec Ref Grid'!C25</f>
+        <v>350</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21335,8 +21453,8 @@
         <v>607</v>
       </c>
       <c r="E168" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B27</f>
-        <v>4200</v>
+        <f aca="false">'1. Elec Ref Grid'!C26</f>
+        <v>500</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21355,8 +21473,8 @@
         <v>607</v>
       </c>
       <c r="E169" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B28</f>
-        <v>2200</v>
+        <f aca="false">'1. Elec Ref Grid'!C27</f>
+        <v>4400</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21375,8 +21493,8 @@
         <v>607</v>
       </c>
       <c r="E170" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B29</f>
-        <v>5772</v>
+        <f aca="false">'1. Elec Ref Grid'!C28</f>
+        <v>4500</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21395,8 +21513,8 @@
         <v>607</v>
       </c>
       <c r="E171" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B30</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C29</f>
+        <v>3110</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21415,8 +21533,8 @@
         <v>607</v>
       </c>
       <c r="E172" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B31</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C30</f>
+        <v>0</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21435,7 +21553,7 @@
         <v>607</v>
       </c>
       <c r="E173" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B32</f>
+        <f aca="false">'1. Elec Ref Grid'!C31</f>
         <v>1000</v>
       </c>
     </row>
@@ -21455,8 +21573,8 @@
         <v>607</v>
       </c>
       <c r="E174" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B33</f>
-        <v>2600</v>
+        <f aca="false">'1. Elec Ref Grid'!C32</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21475,8 +21593,8 @@
         <v>607</v>
       </c>
       <c r="E175" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B34</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C33</f>
+        <v>2500</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21495,8 +21613,8 @@
         <v>607</v>
       </c>
       <c r="E176" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B35</f>
-        <v>1800</v>
+        <f aca="false">'1. Elec Ref Grid'!C34</f>
+        <v>0</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21515,8 +21633,8 @@
         <v>607</v>
       </c>
       <c r="E177" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B36</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C35</f>
+        <v>1100</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21535,8 +21653,8 @@
         <v>607</v>
       </c>
       <c r="E178" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B37</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C36</f>
+        <v>400</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21555,8 +21673,8 @@
         <v>607</v>
       </c>
       <c r="E179" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B38</f>
-        <v>3500</v>
+        <f aca="false">'1. Elec Ref Grid'!C37</f>
+        <v>600</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21575,8 +21693,8 @@
         <v>607</v>
       </c>
       <c r="E180" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B39</f>
-        <v>4800</v>
+        <f aca="false">'1. Elec Ref Grid'!C38</f>
+        <v>3500</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21595,8 +21713,8 @@
         <v>607</v>
       </c>
       <c r="E181" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B40</f>
-        <v>2400</v>
+        <f aca="false">'1. Elec Ref Grid'!C39</f>
+        <v>4800</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21615,8 +21733,8 @@
         <v>607</v>
       </c>
       <c r="E182" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B41</f>
-        <v>1300</v>
+        <f aca="false">'1. Elec Ref Grid'!C40</f>
+        <v>2400</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21635,8 +21753,8 @@
         <v>607</v>
       </c>
       <c r="E183" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B42</f>
-        <v>5000</v>
+        <f aca="false">'1. Elec Ref Grid'!C41</f>
+        <v>1300</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21655,8 +21773,8 @@
         <v>607</v>
       </c>
       <c r="E184" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B43</f>
-        <v>1400</v>
+        <f aca="false">'1. Elec Ref Grid'!C42</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21675,8 +21793,8 @@
         <v>607</v>
       </c>
       <c r="E185" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B44</f>
-        <v>2000</v>
+        <f aca="false">'1. Elec Ref Grid'!C43</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21695,8 +21813,8 @@
         <v>607</v>
       </c>
       <c r="E186" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B45</f>
-        <v>1315</v>
+        <f aca="false">'1. Elec Ref Grid'!C44</f>
+        <v>0</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21715,8 +21833,8 @@
         <v>607</v>
       </c>
       <c r="E187" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B46</f>
-        <v>1400</v>
+        <f aca="false">'1. Elec Ref Grid'!C45</f>
+        <v>1315</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21735,8 +21853,8 @@
         <v>607</v>
       </c>
       <c r="E188" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B47</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C46</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21755,8 +21873,8 @@
         <v>607</v>
       </c>
       <c r="E189" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B48</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C47</f>
+        <v>400</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21775,7 +21893,7 @@
         <v>607</v>
       </c>
       <c r="E190" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B49</f>
+        <f aca="false">'1. Elec Ref Grid'!C48</f>
         <v>600</v>
       </c>
     </row>
@@ -21795,8 +21913,8 @@
         <v>607</v>
       </c>
       <c r="E191" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B50</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C49</f>
+        <v>590</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21815,8 +21933,8 @@
         <v>607</v>
       </c>
       <c r="E192" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B51</f>
-        <v>1700</v>
+        <f aca="false">'1. Elec Ref Grid'!C50</f>
+        <v>0</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21835,8 +21953,8 @@
         <v>607</v>
       </c>
       <c r="E193" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B52</f>
-        <v>700</v>
+        <f aca="false">'1. Elec Ref Grid'!C51</f>
+        <v>1300</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21855,8 +21973,8 @@
         <v>607</v>
       </c>
       <c r="E194" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B53</f>
-        <v>1632</v>
+        <f aca="false">'1. Elec Ref Grid'!C52</f>
+        <v>700</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21875,8 +21993,8 @@
         <v>607</v>
       </c>
       <c r="E195" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B54</f>
-        <v>715</v>
+        <f aca="false">'1. Elec Ref Grid'!C53</f>
+        <v>1632</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21895,8 +22013,8 @@
         <v>607</v>
       </c>
       <c r="E196" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B55</f>
-        <v>1400</v>
+        <f aca="false">'1. Elec Ref Grid'!C54</f>
+        <v>715</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21915,8 +22033,8 @@
         <v>607</v>
       </c>
       <c r="E197" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B56</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C55</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21935,8 +22053,8 @@
         <v>607</v>
       </c>
       <c r="E198" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B57</f>
-        <v>250</v>
+        <f aca="false">'1. Elec Ref Grid'!C56</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21955,8 +22073,8 @@
         <v>607</v>
       </c>
       <c r="E199" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B58</f>
-        <v>1016</v>
+        <f aca="false">'1. Elec Ref Grid'!C57</f>
+        <v>250</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21975,8 +22093,8 @@
         <v>607</v>
       </c>
       <c r="E200" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B59</f>
-        <v>950</v>
+        <f aca="false">'1. Elec Ref Grid'!C58</f>
+        <v>1016</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21995,8 +22113,8 @@
         <v>607</v>
       </c>
       <c r="E201" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B60</f>
-        <v>3000</v>
+        <f aca="false">'1. Elec Ref Grid'!C59</f>
+        <v>879</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22015,8 +22133,8 @@
         <v>607</v>
       </c>
       <c r="E202" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B61</f>
-        <v>240</v>
+        <f aca="false">'1. Elec Ref Grid'!C60</f>
+        <v>3000</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22035,8 +22153,8 @@
         <v>607</v>
       </c>
       <c r="E203" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B62</f>
-        <v>5000</v>
+        <f aca="false">'1. Elec Ref Grid'!C61</f>
+        <v>240</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22055,8 +22173,8 @@
         <v>607</v>
       </c>
       <c r="E204" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B63</f>
-        <v>900</v>
+        <f aca="false">'1. Elec Ref Grid'!C62</f>
+        <v>5000</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22075,8 +22193,8 @@
         <v>607</v>
       </c>
       <c r="E205" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B64</f>
-        <v>4200</v>
+        <f aca="false">'1. Elec Ref Grid'!C63</f>
+        <v>600</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22095,8 +22213,8 @@
         <v>607</v>
       </c>
       <c r="E206" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B65</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C64</f>
+        <v>3500</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22115,8 +22233,8 @@
         <v>607</v>
       </c>
       <c r="E207" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B66</f>
-        <v>2000</v>
+        <f aca="false">'1. Elec Ref Grid'!C65</f>
+        <v>0</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22135,8 +22253,8 @@
         <v>607</v>
       </c>
       <c r="E208" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B67</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C66</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22155,8 +22273,8 @@
         <v>607</v>
       </c>
       <c r="E209" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B68</f>
-        <v>1200</v>
+        <f aca="false">'1. Elec Ref Grid'!C67</f>
+        <v>0</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22175,8 +22293,8 @@
         <v>607</v>
       </c>
       <c r="E210" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B69</f>
-        <v>700</v>
+        <f aca="false">'1. Elec Ref Grid'!C68</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22195,8 +22313,8 @@
         <v>607</v>
       </c>
       <c r="E211" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B70</f>
-        <v>4485</v>
+        <f aca="false">'1. Elec Ref Grid'!C69</f>
+        <v>700</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22215,8 +22333,8 @@
         <v>607</v>
       </c>
       <c r="E212" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B71</f>
-        <v>380</v>
+        <f aca="false">'1. Elec Ref Grid'!C70</f>
+        <v>2160</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22235,8 +22353,8 @@
         <v>607</v>
       </c>
       <c r="E213" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B72</f>
-        <v>5600</v>
+        <f aca="false">'1. Elec Ref Grid'!C71</f>
+        <v>0</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22255,8 +22373,8 @@
         <v>607</v>
       </c>
       <c r="E214" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B73</f>
-        <v>120</v>
+        <f aca="false">'1. Elec Ref Grid'!C72</f>
+        <v>5600</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22275,8 +22393,8 @@
         <v>607</v>
       </c>
       <c r="E215" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B74</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C73</f>
+        <v>150</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22295,8 +22413,8 @@
         <v>607</v>
       </c>
       <c r="E216" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B75</f>
-        <v>500</v>
+        <f aca="false">'1. Elec Ref Grid'!C74</f>
+        <v>800</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22315,8 +22433,8 @@
         <v>607</v>
       </c>
       <c r="E217" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B76</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C75</f>
+        <v>500</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22335,8 +22453,8 @@
         <v>607</v>
       </c>
       <c r="E218" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B77</f>
-        <v>1100</v>
+        <f aca="false">'1. Elec Ref Grid'!C76</f>
+        <v>0</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22355,8 +22473,8 @@
         <v>607</v>
       </c>
       <c r="E219" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B78</f>
-        <v>660</v>
+        <f aca="false">'1. Elec Ref Grid'!C77</f>
+        <v>850</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22375,8 +22493,8 @@
         <v>607</v>
       </c>
       <c r="E220" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B79</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C78</f>
+        <v>580</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22395,8 +22513,8 @@
         <v>607</v>
       </c>
       <c r="E221" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B80</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C79</f>
+        <v>0</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22415,8 +22533,8 @@
         <v>607</v>
       </c>
       <c r="E222" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B81</f>
-        <v>300</v>
+        <f aca="false">'1. Elec Ref Grid'!C80</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22435,8 +22553,8 @@
         <v>607</v>
       </c>
       <c r="E223" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B82</f>
-        <v>1500</v>
+        <f aca="false">'1. Elec Ref Grid'!C81</f>
+        <v>400</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22455,8 +22573,8 @@
         <v>607</v>
       </c>
       <c r="E224" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B83</f>
-        <v>1617</v>
+        <f aca="false">'1. Elec Ref Grid'!C82</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22475,8 +22593,8 @@
         <v>607</v>
       </c>
       <c r="E225" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B84</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C83</f>
+        <v>1435</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22495,8 +22613,8 @@
         <v>607</v>
       </c>
       <c r="E226" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B85</f>
-        <v>1200</v>
+        <f aca="false">'1. Elec Ref Grid'!C84</f>
+        <v>700</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22515,8 +22633,8 @@
         <v>607</v>
       </c>
       <c r="E227" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B86</f>
-        <v>1800</v>
+        <f aca="false">'1. Elec Ref Grid'!C85</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22535,8 +22653,8 @@
         <v>607</v>
       </c>
       <c r="E228" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B87</f>
-        <v>450</v>
+        <f aca="false">'1. Elec Ref Grid'!C86</f>
+        <v>2513</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22555,8 +22673,8 @@
         <v>607</v>
       </c>
       <c r="E229" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B88</f>
-        <v>1750</v>
+        <f aca="false">'1. Elec Ref Grid'!C87</f>
+        <v>650</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22575,8 +22693,8 @@
         <v>607</v>
       </c>
       <c r="E230" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B89</f>
-        <v>1250</v>
+        <f aca="false">'1. Elec Ref Grid'!C88</f>
+        <v>1750</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22595,8 +22713,8 @@
         <v>607</v>
       </c>
       <c r="E231" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B90</f>
-        <v>3000</v>
+        <f aca="false">'1. Elec Ref Grid'!C89</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22615,8 +22733,8 @@
         <v>607</v>
       </c>
       <c r="E232" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B91</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C90</f>
+        <v>3000</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22635,8 +22753,8 @@
         <v>607</v>
       </c>
       <c r="E233" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B92</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C91</f>
+        <v>0</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22655,8 +22773,8 @@
         <v>607</v>
       </c>
       <c r="E234" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B93</f>
-        <v>4650</v>
+        <f aca="false">'1. Elec Ref Grid'!C92</f>
+        <v>400</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22675,8 +22793,8 @@
         <v>607</v>
       </c>
       <c r="E235" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B94</f>
-        <v>4500</v>
+        <f aca="false">'1. Elec Ref Grid'!C93</f>
+        <v>5350</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22695,8 +22813,8 @@
         <v>607</v>
       </c>
       <c r="E236" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B95</f>
-        <v>420</v>
+        <f aca="false">'1. Elec Ref Grid'!C94</f>
+        <v>5300</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22715,8 +22833,8 @@
         <v>607</v>
       </c>
       <c r="E237" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B96</f>
-        <v>3100</v>
+        <f aca="false">'1. Elec Ref Grid'!C95</f>
+        <v>480</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22735,8 +22853,8 @@
         <v>607</v>
       </c>
       <c r="E238" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B97</f>
-        <v>720</v>
+        <f aca="false">'1. Elec Ref Grid'!C96</f>
+        <v>5700</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22755,8 +22873,8 @@
         <v>607</v>
       </c>
       <c r="E239" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B98</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C97</f>
+        <v>900</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22775,8 +22893,8 @@
         <v>607</v>
       </c>
       <c r="E240" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B99</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C98</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22795,8 +22913,8 @@
         <v>607</v>
       </c>
       <c r="E241" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B100</f>
-        <v>1080</v>
+        <f aca="false">'1. Elec Ref Grid'!C99</f>
+        <v>600</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22815,8 +22933,8 @@
         <v>607</v>
       </c>
       <c r="E242" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B101</f>
-        <v>2000</v>
+        <f aca="false">'1. Elec Ref Grid'!C100</f>
+        <v>1153</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22835,8 +22953,8 @@
         <v>607</v>
       </c>
       <c r="E243" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B102</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C101</f>
+        <v>3250</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22855,8 +22973,8 @@
         <v>607</v>
       </c>
       <c r="E244" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B103</f>
-        <v>2000</v>
+        <f aca="false">'1. Elec Ref Grid'!C102</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22875,8 +22993,8 @@
         <v>607</v>
       </c>
       <c r="E245" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B104</f>
-        <v>1500</v>
+        <f aca="false">'1. Elec Ref Grid'!C103</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22895,8 +23013,8 @@
         <v>607</v>
       </c>
       <c r="E246" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B105</f>
-        <v>225</v>
+        <f aca="false">'1. Elec Ref Grid'!C104</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22915,8 +23033,8 @@
         <v>607</v>
       </c>
       <c r="E247" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B106</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C105</f>
+        <v>225</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22935,8 +23053,8 @@
         <v>607</v>
       </c>
       <c r="E248" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B107</f>
-        <v>950</v>
+        <f aca="false">'1. Elec Ref Grid'!C106</f>
+        <v>600</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22955,8 +23073,8 @@
         <v>607</v>
       </c>
       <c r="E249" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B108</f>
-        <v>700</v>
+        <f aca="false">'1. Elec Ref Grid'!C107</f>
+        <v>950</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22975,7 +23093,7 @@
         <v>607</v>
       </c>
       <c r="E250" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B109</f>
+        <f aca="false">'1. Elec Ref Grid'!C108</f>
         <v>700</v>
       </c>
     </row>
@@ -22995,8 +23113,8 @@
         <v>607</v>
       </c>
       <c r="E251" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B110</f>
-        <v>500</v>
+        <f aca="false">'1. Elec Ref Grid'!C109</f>
+        <v>700</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23015,8 +23133,8 @@
         <v>607</v>
       </c>
       <c r="E252" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B111</f>
-        <v>540</v>
+        <f aca="false">'1. Elec Ref Grid'!C110</f>
+        <v>500</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23035,8 +23153,8 @@
         <v>607</v>
       </c>
       <c r="E253" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B112</f>
-        <v>460</v>
+        <f aca="false">'1. Elec Ref Grid'!C111</f>
+        <v>1140</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23055,8 +23173,8 @@
         <v>607</v>
       </c>
       <c r="E254" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B113</f>
-        <v>700</v>
+        <f aca="false">'1. Elec Ref Grid'!C112</f>
+        <v>480</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23075,8 +23193,8 @@
         <v>607</v>
       </c>
       <c r="E255" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B114</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C113</f>
+        <v>700</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23095,8 +23213,8 @@
         <v>607</v>
       </c>
       <c r="E256" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B115</f>
-        <v>350</v>
+        <f aca="false">'1. Elec Ref Grid'!C114</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23115,8 +23233,8 @@
         <v>607</v>
       </c>
       <c r="E257" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B116</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C115</f>
+        <v>1300</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23135,7 +23253,7 @@
         <v>607</v>
       </c>
       <c r="E258" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B117</f>
+        <f aca="false">'1. Elec Ref Grid'!C116</f>
         <v>600</v>
       </c>
     </row>
@@ -23155,8 +23273,8 @@
         <v>607</v>
       </c>
       <c r="E259" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B118</f>
-        <v>700</v>
+        <f aca="false">'1. Elec Ref Grid'!C117</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23175,8 +23293,8 @@
         <v>607</v>
       </c>
       <c r="E260" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B119</f>
-        <v>250</v>
+        <f aca="false">'1. Elec Ref Grid'!C118</f>
+        <v>600</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23195,8 +23313,8 @@
         <v>607</v>
       </c>
       <c r="E261" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B120</f>
-        <v>2145</v>
+        <f aca="false">'1. Elec Ref Grid'!C119</f>
+        <v>300</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23215,8 +23333,8 @@
         <v>607</v>
       </c>
       <c r="E262" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B121</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C120</f>
+        <v>2095</v>
       </c>
     </row>
     <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23235,8 +23353,8 @@
         <v>607</v>
       </c>
       <c r="E263" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B122</f>
-        <v>3000</v>
+        <f aca="false">'1. Elec Ref Grid'!C121</f>
+        <v>0</v>
       </c>
     </row>
     <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23255,8 +23373,8 @@
         <v>607</v>
       </c>
       <c r="E264" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B123</f>
-        <v>781</v>
+        <f aca="false">'1. Elec Ref Grid'!C122</f>
+        <v>0</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23275,8 +23393,8 @@
         <v>607</v>
       </c>
       <c r="E265" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B124</f>
-        <v>3000</v>
+        <f aca="false">'1. Elec Ref Grid'!C123</f>
+        <v>0</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23295,8 +23413,8 @@
         <v>607</v>
       </c>
       <c r="E266" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B125</f>
-        <v>3000</v>
+        <f aca="false">'1. Elec Ref Grid'!C124</f>
+        <v>0</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23315,8 +23433,8 @@
         <v>607</v>
       </c>
       <c r="E267" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B126</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C125</f>
+        <v>0</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23335,8 +23453,8 @@
         <v>607</v>
       </c>
       <c r="E268" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B127</f>
-        <v>1984</v>
+        <f aca="false">'1. Elec Ref Grid'!C126</f>
+        <v>600</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23355,8 +23473,8 @@
         <v>607</v>
       </c>
       <c r="E269" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B128</f>
-        <v>150</v>
+        <f aca="false">'1. Elec Ref Grid'!C127</f>
+        <v>1800</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23375,8 +23493,8 @@
         <v>607</v>
       </c>
       <c r="E270" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B129</f>
-        <v>3300</v>
+        <f aca="false">'1. Elec Ref Grid'!C128</f>
+        <v>150</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23395,8 +23513,8 @@
         <v>607</v>
       </c>
       <c r="E271" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B130</f>
-        <v>7300</v>
+        <f aca="false">'1. Elec Ref Grid'!C129</f>
+        <v>3300</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23415,8 +23533,8 @@
         <v>607</v>
       </c>
       <c r="E272" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B131</f>
-        <v>6200</v>
+        <f aca="false">'1. Elec Ref Grid'!C130</f>
+        <v>7300</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23435,8 +23553,8 @@
         <v>607</v>
       </c>
       <c r="E273" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B132</f>
-        <v>818</v>
+        <f aca="false">'1. Elec Ref Grid'!C131</f>
+        <v>2800</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23455,8 +23573,8 @@
         <v>607</v>
       </c>
       <c r="E274" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B133</f>
-        <v>495</v>
+        <f aca="false">'1. Elec Ref Grid'!C132</f>
+        <v>0</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23475,8 +23593,8 @@
         <v>607</v>
       </c>
       <c r="E275" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B134</f>
-        <v>1400</v>
+        <f aca="false">'1. Elec Ref Grid'!C133</f>
+        <v>634</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23495,8 +23613,8 @@
         <v>607</v>
       </c>
       <c r="E276" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B135</f>
-        <v>450</v>
+        <f aca="false">'1. Elec Ref Grid'!C134</f>
+        <v>1400</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23515,8 +23633,8 @@
         <v>607</v>
       </c>
       <c r="E277" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B136</f>
-        <v>480</v>
+        <f aca="false">'1. Elec Ref Grid'!C135</f>
+        <v>400</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23535,8 +23653,8 @@
         <v>607</v>
       </c>
       <c r="E278" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B137</f>
-        <v>2000</v>
+        <f aca="false">'1. Elec Ref Grid'!C136</f>
+        <v>950</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23555,8 +23673,8 @@
         <v>607</v>
       </c>
       <c r="E279" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B138</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C137</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23575,8 +23693,8 @@
         <v>607</v>
       </c>
       <c r="E280" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B139</f>
-        <v>1000</v>
+        <f aca="false">'1. Elec Ref Grid'!C138</f>
+        <v>0</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23595,8 +23713,8 @@
         <v>607</v>
       </c>
       <c r="E281" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B140</f>
-        <v>500</v>
+        <f aca="false">'1. Elec Ref Grid'!C139</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23615,8 +23733,8 @@
         <v>607</v>
       </c>
       <c r="E282" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B141</f>
-        <v>800</v>
+        <f aca="false">'1. Elec Ref Grid'!C140</f>
+        <v>500</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23635,8 +23753,8 @@
         <v>607</v>
       </c>
       <c r="E283" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B142</f>
-        <v>400</v>
+        <f aca="false">'1. Elec Ref Grid'!C141</f>
+        <v>800</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23655,8 +23773,8 @@
         <v>607</v>
       </c>
       <c r="E284" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B143</f>
-        <v>600</v>
+        <f aca="false">'1. Elec Ref Grid'!C142</f>
+        <v>400</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23675,8 +23793,8 @@
         <v>607</v>
       </c>
       <c r="E285" s="1" t="n">
-        <f aca="false">'1. Elec Ref Grid'!B144</f>
-        <v>0</v>
+        <f aca="false">'1. Elec Ref Grid'!C143</f>
+        <v>600</v>
       </c>
     </row>
     <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28186,7 +28304,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A2,LEN('2. H2 Ref Grid'!A2)-FIND("-",'2. H2 Ref Grid'!A2))</f>
         <v>DE</v>
       </c>
-      <c r="B37" s="17" t="str">
+      <c r="B37" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A2,FIND("-",'2. H2 Ref Grid'!A2)-1)</f>
         <v>AT</v>
       </c>
@@ -28205,7 +28323,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A3,LEN('2. H2 Ref Grid'!A3)-FIND("-",'2. H2 Ref Grid'!A3))</f>
         <v>IBIT</v>
       </c>
-      <c r="B38" s="17" t="str">
+      <c r="B38" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A3,FIND("-",'2. H2 Ref Grid'!A3)-1)</f>
         <v>AT</v>
       </c>
@@ -28224,7 +28342,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A4,LEN('2. H2 Ref Grid'!A4)-FIND("-",'2. H2 Ref Grid'!A4))</f>
         <v>SI</v>
       </c>
-      <c r="B39" s="17" t="str">
+      <c r="B39" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A4,FIND("-",'2. H2 Ref Grid'!A4)-1)</f>
         <v>AT</v>
       </c>
@@ -28243,7 +28361,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A5,LEN('2. H2 Ref Grid'!A5)-FIND("-",'2. H2 Ref Grid'!A5))</f>
         <v>SK</v>
       </c>
-      <c r="B40" s="17" t="str">
+      <c r="B40" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A5,FIND("-",'2. H2 Ref Grid'!A5)-1)</f>
         <v>AT</v>
       </c>
@@ -28262,7 +28380,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A6,LEN('2. H2 Ref Grid'!A6)-FIND("-",'2. H2 Ref Grid'!A6))</f>
         <v>DE</v>
       </c>
-      <c r="B41" s="17" t="str">
+      <c r="B41" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A6,FIND("-",'2. H2 Ref Grid'!A6)-1)</f>
         <v>BE</v>
       </c>
@@ -28281,7 +28399,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A7,LEN('2. H2 Ref Grid'!A7)-FIND("-",'2. H2 Ref Grid'!A7))</f>
         <v>FR</v>
       </c>
-      <c r="B42" s="17" t="str">
+      <c r="B42" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A7,FIND("-",'2. H2 Ref Grid'!A7)-1)</f>
         <v>BE</v>
       </c>
@@ -28300,7 +28418,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A8,LEN('2. H2 Ref Grid'!A8)-FIND("-",'2. H2 Ref Grid'!A8))</f>
         <v>LU</v>
       </c>
-      <c r="B43" s="17" t="str">
+      <c r="B43" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A8,FIND("-",'2. H2 Ref Grid'!A8)-1)</f>
         <v>BE</v>
       </c>
@@ -28319,7 +28437,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A9,LEN('2. H2 Ref Grid'!A9)-FIND("-",'2. H2 Ref Grid'!A9))</f>
         <v>NL</v>
       </c>
-      <c r="B44" s="17" t="str">
+      <c r="B44" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A9,FIND("-",'2. H2 Ref Grid'!A9)-1)</f>
         <v>BE</v>
       </c>
@@ -28338,7 +28456,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A10,LEN('2. H2 Ref Grid'!A10)-FIND("-",'2. H2 Ref Grid'!A10))</f>
         <v>GR</v>
       </c>
-      <c r="B45" s="17" t="str">
+      <c r="B45" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A10,FIND("-",'2. H2 Ref Grid'!A10)-1)</f>
         <v>BG</v>
       </c>
@@ -28357,7 +28475,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A11,LEN('2. H2 Ref Grid'!A11)-FIND("-",'2. H2 Ref Grid'!A11))</f>
         <v>RO</v>
       </c>
-      <c r="B46" s="17" t="str">
+      <c r="B46" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A11,FIND("-",'2. H2 Ref Grid'!A11)-1)</f>
         <v>BG</v>
       </c>
@@ -28376,7 +28494,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A12,LEN('2. H2 Ref Grid'!A12)-FIND("-",'2. H2 Ref Grid'!A12))</f>
         <v>IBIT</v>
       </c>
-      <c r="B47" s="17" t="str">
+      <c r="B47" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A12,FIND("-",'2. H2 Ref Grid'!A12)-1)</f>
         <v>CH</v>
       </c>
@@ -28395,7 +28513,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A13,LEN('2. H2 Ref Grid'!A13)-FIND("-",'2. H2 Ref Grid'!A13))</f>
         <v>DE</v>
       </c>
-      <c r="B48" s="17" t="str">
+      <c r="B48" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A13,FIND("-",'2. H2 Ref Grid'!A13)-1)</f>
         <v>CZ</v>
       </c>
@@ -28414,7 +28532,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A14,LEN('2. H2 Ref Grid'!A14)-FIND("-",'2. H2 Ref Grid'!A14))</f>
         <v>DK</v>
       </c>
-      <c r="B49" s="17" t="str">
+      <c r="B49" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A14,FIND("-",'2. H2 Ref Grid'!A14)-1)</f>
         <v>DE</v>
       </c>
@@ -28433,7 +28551,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A15,LEN('2. H2 Ref Grid'!A15)-FIND("-",'2. H2 Ref Grid'!A15))</f>
         <v>FR</v>
       </c>
-      <c r="B50" s="17" t="str">
+      <c r="B50" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A15,FIND("-",'2. H2 Ref Grid'!A15)-1)</f>
         <v>DE</v>
       </c>
@@ -28452,7 +28570,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A16,LEN('2. H2 Ref Grid'!A16)-FIND("-",'2. H2 Ref Grid'!A16))</f>
         <v>NL</v>
       </c>
-      <c r="B51" s="17" t="str">
+      <c r="B51" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A16,FIND("-",'2. H2 Ref Grid'!A16)-1)</f>
         <v>DE</v>
       </c>
@@ -28471,7 +28589,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A17,LEN('2. H2 Ref Grid'!A17)-FIND("-",'2. H2 Ref Grid'!A17))</f>
         <v>PL</v>
       </c>
-      <c r="B52" s="17" t="str">
+      <c r="B52" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A17,FIND("-",'2. H2 Ref Grid'!A17)-1)</f>
         <v>DE</v>
       </c>
@@ -28490,7 +28608,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A18,LEN('2. H2 Ref Grid'!A18)-FIND("-",'2. H2 Ref Grid'!A18))</f>
         <v>FI</v>
       </c>
-      <c r="B53" s="17" t="str">
+      <c r="B53" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A18,FIND("-",'2. H2 Ref Grid'!A18)-1)</f>
         <v>EE</v>
       </c>
@@ -28509,7 +28627,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A19,LEN('2. H2 Ref Grid'!A19)-FIND("-",'2. H2 Ref Grid'!A19))</f>
         <v>LV</v>
       </c>
-      <c r="B54" s="17" t="str">
+      <c r="B54" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A19,FIND("-",'2. H2 Ref Grid'!A19)-1)</f>
         <v>EE</v>
       </c>
@@ -28528,7 +28646,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A20,LEN('2. H2 Ref Grid'!A20)-FIND("-",'2. H2 Ref Grid'!A20))</f>
         <v>FR</v>
       </c>
-      <c r="B55" s="17" t="str">
+      <c r="B55" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A20,FIND("-",'2. H2 Ref Grid'!A20)-1)</f>
         <v>ES</v>
       </c>
@@ -28547,7 +28665,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A21,LEN('2. H2 Ref Grid'!A21)-FIND("-",'2. H2 Ref Grid'!A21))</f>
         <v>IT</v>
       </c>
-      <c r="B56" s="17" t="str">
+      <c r="B56" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A21,FIND("-",'2. H2 Ref Grid'!A21)-1)</f>
         <v>ES</v>
       </c>
@@ -28566,7 +28684,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A22,LEN('2. H2 Ref Grid'!A22)-FIND("-",'2. H2 Ref Grid'!A22))</f>
         <v>PT</v>
       </c>
-      <c r="B57" s="17" t="str">
+      <c r="B57" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A22,FIND("-",'2. H2 Ref Grid'!A22)-1)</f>
         <v>ES</v>
       </c>
@@ -28585,7 +28703,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A23,LEN('2. H2 Ref Grid'!A23)-FIND("-",'2. H2 Ref Grid'!A23))</f>
         <v>SE</v>
       </c>
-      <c r="B58" s="17" t="str">
+      <c r="B58" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A23,FIND("-",'2. H2 Ref Grid'!A23)-1)</f>
         <v>FI</v>
       </c>
@@ -28604,7 +28722,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A24,LEN('2. H2 Ref Grid'!A24)-FIND("-",'2. H2 Ref Grid'!A24))</f>
         <v>HU</v>
       </c>
-      <c r="B59" s="17" t="str">
+      <c r="B59" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A24,FIND("-",'2. H2 Ref Grid'!A24)-1)</f>
         <v>HR</v>
       </c>
@@ -28623,7 +28741,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A25,LEN('2. H2 Ref Grid'!A25)-FIND("-",'2. H2 Ref Grid'!A25))</f>
         <v>SI</v>
       </c>
-      <c r="B60" s="17" t="str">
+      <c r="B60" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A25,FIND("-",'2. H2 Ref Grid'!A25)-1)</f>
         <v>HR</v>
       </c>
@@ -28642,7 +28760,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A26,LEN('2. H2 Ref Grid'!A26)-FIND("-",'2. H2 Ref Grid'!A26))</f>
         <v>RO</v>
       </c>
-      <c r="B61" s="17" t="str">
+      <c r="B61" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A26,FIND("-",'2. H2 Ref Grid'!A26)-1)</f>
         <v>HU</v>
       </c>
@@ -28661,7 +28779,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A27,LEN('2. H2 Ref Grid'!A27)-FIND("-",'2. H2 Ref Grid'!A27))</f>
         <v>SI</v>
       </c>
-      <c r="B62" s="17" t="str">
+      <c r="B62" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A27,FIND("-",'2. H2 Ref Grid'!A27)-1)</f>
         <v>HU</v>
       </c>
@@ -28680,7 +28798,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A28,LEN('2. H2 Ref Grid'!A28)-FIND("-",'2. H2 Ref Grid'!A28))</f>
         <v>SK</v>
       </c>
-      <c r="B63" s="17" t="str">
+      <c r="B63" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A28,FIND("-",'2. H2 Ref Grid'!A28)-1)</f>
         <v>HU</v>
       </c>
@@ -28699,7 +28817,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A29,LEN('2. H2 Ref Grid'!A29)-FIND("-",'2. H2 Ref Grid'!A29))</f>
         <v>SI</v>
       </c>
-      <c r="B64" s="17" t="str">
+      <c r="B64" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A29,FIND("-",'2. H2 Ref Grid'!A29)-1)</f>
         <v>IT</v>
       </c>
@@ -28718,7 +28836,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A30,LEN('2. H2 Ref Grid'!A30)-FIND("-",'2. H2 Ref Grid'!A30))</f>
         <v>LV</v>
       </c>
-      <c r="B65" s="17" t="str">
+      <c r="B65" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A30,FIND("-",'2. H2 Ref Grid'!A30)-1)</f>
         <v>LT</v>
       </c>
@@ -28737,7 +28855,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A31,LEN('2. H2 Ref Grid'!A31)-FIND("-",'2. H2 Ref Grid'!A31))</f>
         <v>PL</v>
       </c>
-      <c r="B66" s="17" t="str">
+      <c r="B66" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A31,FIND("-",'2. H2 Ref Grid'!A31)-1)</f>
         <v>LT</v>
       </c>
@@ -28756,7 +28874,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A32,LEN('2. H2 Ref Grid'!A32)-FIND("-",'2. H2 Ref Grid'!A32))</f>
         <v>CZ</v>
       </c>
-      <c r="B67" s="17" t="str">
+      <c r="B67" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A32,FIND("-",'2. H2 Ref Grid'!A32)-1)</f>
         <v>SK</v>
       </c>
@@ -28775,7 +28893,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A33,LEN('2. H2 Ref Grid'!A33)-FIND("-",'2. H2 Ref Grid'!A33))</f>
         <v>IBFI</v>
       </c>
-      <c r="B68" s="17" t="str">
+      <c r="B68" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A33,FIND("-",'2. H2 Ref Grid'!A33)-1)</f>
         <v>FI</v>
       </c>
@@ -28794,7 +28912,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A34,LEN('2. H2 Ref Grid'!A34)-FIND("-",'2. H2 Ref Grid'!A34))</f>
         <v>IBFI</v>
       </c>
-      <c r="B69" s="17" t="str">
+      <c r="B69" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A34,FIND("-",'2. H2 Ref Grid'!A34)-1)</f>
         <v>SE</v>
       </c>
@@ -28813,7 +28931,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A35,LEN('2. H2 Ref Grid'!A35)-FIND("-",'2. H2 Ref Grid'!A35))</f>
         <v>IBIT</v>
       </c>
-      <c r="B70" s="17" t="str">
+      <c r="B70" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A35,FIND("-",'2. H2 Ref Grid'!A35)-1)</f>
         <v>IT</v>
       </c>
@@ -28832,7 +28950,7 @@
         <f aca="false">RIGHT('2. H2 Ref Grid'!A36,LEN('2. H2 Ref Grid'!A36)-FIND("-",'2. H2 Ref Grid'!A36))</f>
         <v>IBFI</v>
       </c>
-      <c r="B71" s="17" t="str">
+      <c r="B71" s="12" t="str">
         <f aca="false">LEFT('2. H2 Ref Grid'!A36,FIND("-",'2. H2 Ref Grid'!A36)-1)</f>
         <v>DE</v>
       </c>

</xml_diff>